<commit_message>
E2E artefacts from the in-progress full sweep
Screenshots and generated upload workbooks from the first scripts of the
48-script re-run. Artefacts only — 33 PNGs and 4 XLSX files, nothing
outside e2e-screenshots/.

The four accessory workbooks are the meaningful ones. They are now built
by addressing columns by header name rather than by position, so the
committed files carry the buy and sale prices in BP and SP instead of
leaving those cells empty and spilling the supplier into Model. Committed
mid-sweep because the run is long and the container has reset repeatedly
today; the remainder follows when it finishes.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01T4LurPsVU5WNa1i8str9pz
</commit_message>
<xml_diff>
--- a/e2e-screenshots/accessory-visibility/sales-accessory-1.xlsx
+++ b/e2e-screenshots/accessory-visibility/sales-accessory-1.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="53">
   <si>
     <t>Date</t>
   </si>
@@ -746,7 +746,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>31</v>
       </c>
@@ -759,38 +759,20 @@
       <c r="D2" t="s">
         <v>34</v>
       </c>
-      <c r="E2" t="s">
+      <c r="H2" t="s">
         <v>35</v>
       </c>
-      <c r="F2">
+      <c r="I2">
         <v>2</v>
       </c>
-      <c r="G2">
+      <c r="J2">
         <v>3.5</v>
       </c>
-      <c r="H2">
+      <c r="K2">
         <v>8.99</v>
       </c>
-      <c r="I2" t="s">
-        <v>34</v>
-      </c>
-      <c r="J2" t="s">
-        <v>34</v>
-      </c>
-      <c r="K2" t="s">
-        <v>34</v>
-      </c>
-      <c r="L2">
+      <c r="R2">
         <v>0</v>
-      </c>
-      <c r="M2" t="s">
-        <v>34</v>
-      </c>
-      <c r="N2" t="s">
-        <v>34</v>
-      </c>
-      <c r="O2" t="s">
-        <v>34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>